<commit_message>
25 Companies Added in the substack feed.
</commit_message>
<xml_diff>
--- a/source_links.xlsx
+++ b/source_links.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RCK Analytics\Development\insider_monkey_article_scraping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Insider Monkey\insider-monkey-substacks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53D62979-D398-4686-939C-68E510788A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0394C52-F490-4057-8F08-1B2543532677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Twitter" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="814">
   <si>
     <t>Sr No.</t>
   </si>
@@ -2328,6 +2328,156 @@
   </si>
   <si>
     <t>https://www.worldstocksinvestment.com/archive</t>
+  </si>
+  <si>
+    <t>Adaptive Asset Analytics</t>
+  </si>
+  <si>
+    <t>https://adamniedbalski.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Aesop Investment Research</t>
+  </si>
+  <si>
+    <t>https://medismarketnotes.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Arbor Terminal</t>
+  </si>
+  <si>
+    <t>https://elmwoodinvestor.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Capital Blueprint</t>
+  </si>
+  <si>
+    <t>https://capitalblueprint.substack.com/archive</t>
+  </si>
+  <si>
+    <t>ChartWaveInvesting's Substack</t>
+  </si>
+  <si>
+    <t>https://chartwaveinvesting.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Dengler Deep Dives</t>
+  </si>
+  <si>
+    <t>https://ryandengler.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Equity Empire</t>
+  </si>
+  <si>
+    <t>https://theinvestorchannel.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Financial Reports Made Simple</t>
+  </si>
+  <si>
+    <t>https://financialreportsmadesimple.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Finimize Analyst Desk</t>
+  </si>
+  <si>
+    <t>https://finimize.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Glocal Investor</t>
+  </si>
+  <si>
+    <t>https://glocalinvestor.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Growth Dragons</t>
+  </si>
+  <si>
+    <t>https://growthdragons.substack.com/archive?sort=new</t>
+  </si>
+  <si>
+    <t>Inelastic Models</t>
+  </si>
+  <si>
+    <t>https://inelasticmodels.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Intern Pierre</t>
+  </si>
+  <si>
+    <t>https://internpierre.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Jorgen</t>
+  </si>
+  <si>
+    <t>https://topcornerinvesting.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Komodo Capital</t>
+  </si>
+  <si>
+    <t>https://komodocapital.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Markman Capital Insight</t>
+  </si>
+  <si>
+    <t>https://markmancapitalinsight.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Outside The Index</t>
+  </si>
+  <si>
+    <t>https://outsidetheindex.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Secondary Scoop</t>
+  </si>
+  <si>
+    <t>https://www.secondaryscoop.com/archive</t>
+  </si>
+  <si>
+    <t>Stock Reports &amp; Analysis</t>
+  </si>
+  <si>
+    <t>https://wealthmatica.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Stock Talk Newsletter</t>
+  </si>
+  <si>
+    <t>https://stocktalknewsletter.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Substack on StockCompass</t>
+  </si>
+  <si>
+    <t>https://stockcompass.substack.com/archive</t>
+  </si>
+  <si>
+    <t>TheDividendPrince</t>
+  </si>
+  <si>
+    <t>https://thedividendprince.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Thesis Rationale</t>
+  </si>
+  <si>
+    <t>https://thesisrationale.substack.com/archive</t>
+  </si>
+  <si>
+    <t>TuDi's F.L.O.W. INVESTING Method</t>
+  </si>
+  <si>
+    <t>https://stockflowmethod.substack.com/archive</t>
+  </si>
+  <si>
+    <t>Value Investing</t>
+  </si>
+  <si>
+    <t>https://valueoverhype.substack.com/archive</t>
   </si>
 </sst>
 </file>
@@ -2692,14 +2842,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:D13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -2710,7 +2860,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -2721,7 +2871,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>2</v>
       </c>
@@ -2732,7 +2882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>3</v>
       </c>
@@ -2743,7 +2893,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>4</v>
       </c>
@@ -2754,7 +2904,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>5</v>
       </c>
@@ -2765,7 +2915,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>6</v>
       </c>
@@ -2776,27 +2926,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>11</v>
       </c>
@@ -2816,14 +2966,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA25BD73-CCC7-4112-B82B-D24C1210E61D}">
-  <dimension ref="A1:B381"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B406"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -2831,7 +2981,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
@@ -2839,7 +2989,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
@@ -2847,7 +2997,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
@@ -2855,7 +3005,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
@@ -2863,7 +3013,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
@@ -2871,7 +3021,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>27</v>
       </c>
@@ -2879,7 +3029,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>28</v>
       </c>
@@ -2887,7 +3037,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>31</v>
       </c>
@@ -2895,7 +3045,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>32</v>
       </c>
@@ -2903,7 +3053,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
@@ -2911,7 +3061,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>34</v>
       </c>
@@ -2919,7 +3069,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>39</v>
       </c>
@@ -2927,7 +3077,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>40</v>
       </c>
@@ -2935,7 +3085,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>41</v>
       </c>
@@ -2943,7 +3093,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>42</v>
       </c>
@@ -2951,7 +3101,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
@@ -2959,7 +3109,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>44</v>
       </c>
@@ -2967,7 +3117,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>45</v>
       </c>
@@ -2975,7 +3125,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>46</v>
       </c>
@@ -2983,7 +3133,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>47</v>
       </c>
@@ -2991,7 +3141,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>48</v>
       </c>
@@ -2999,7 +3149,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>49</v>
       </c>
@@ -3007,7 +3157,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>50</v>
       </c>
@@ -3015,7 +3165,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>51</v>
       </c>
@@ -3023,7 +3173,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>52</v>
       </c>
@@ -3031,7 +3181,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>55</v>
       </c>
@@ -3039,7 +3189,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>56</v>
       </c>
@@ -3047,7 +3197,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>57</v>
       </c>
@@ -3055,7 +3205,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>70</v>
       </c>
@@ -3063,7 +3213,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>60</v>
       </c>
@@ -3071,7 +3221,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>61</v>
       </c>
@@ -3079,7 +3229,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>62</v>
       </c>
@@ -3087,7 +3237,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>63</v>
       </c>
@@ -3095,7 +3245,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>68</v>
       </c>
@@ -3103,7 +3253,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>69</v>
       </c>
@@ -3111,7 +3261,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>71</v>
       </c>
@@ -3119,7 +3269,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>72</v>
       </c>
@@ -3127,7 +3277,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>73</v>
       </c>
@@ -3135,7 +3285,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>74</v>
       </c>
@@ -3143,7 +3293,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>75</v>
       </c>
@@ -3151,7 +3301,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>76</v>
       </c>
@@ -3159,7 +3309,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>77</v>
       </c>
@@ -3167,7 +3317,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>78</v>
       </c>
@@ -3175,7 +3325,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>83</v>
       </c>
@@ -3183,7 +3333,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>84</v>
       </c>
@@ -3191,7 +3341,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>85</v>
       </c>
@@ -3199,7 +3349,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>86</v>
       </c>
@@ -3207,7 +3357,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>89</v>
       </c>
@@ -3215,7 +3365,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>90</v>
       </c>
@@ -3223,7 +3373,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>91</v>
       </c>
@@ -3231,7 +3381,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>92</v>
       </c>
@@ -3239,7 +3389,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>93</v>
       </c>
@@ -3247,7 +3397,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>94</v>
       </c>
@@ -3255,7 +3405,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>97</v>
       </c>
@@ -3263,7 +3413,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>98</v>
       </c>
@@ -3271,7 +3421,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>101</v>
       </c>
@@ -3279,7 +3429,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>105</v>
       </c>
@@ -3287,7 +3437,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>106</v>
       </c>
@@ -3295,7 +3445,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>107</v>
       </c>
@@ -3303,7 +3453,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>108</v>
       </c>
@@ -3311,7 +3461,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>109</v>
       </c>
@@ -3319,7 +3469,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>112</v>
       </c>
@@ -3327,7 +3477,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>113</v>
       </c>
@@ -3335,7 +3485,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>114</v>
       </c>
@@ -3343,7 +3493,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>115</v>
       </c>
@@ -3351,7 +3501,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>118</v>
       </c>
@@ -3359,7 +3509,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>119</v>
       </c>
@@ -3367,7 +3517,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>120</v>
       </c>
@@ -3375,7 +3525,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>122</v>
       </c>
@@ -3383,7 +3533,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>123</v>
       </c>
@@ -3391,7 +3541,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>124</v>
       </c>
@@ -3399,7 +3549,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>125</v>
       </c>
@@ -3407,7 +3557,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>126</v>
       </c>
@@ -3415,7 +3565,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>127</v>
       </c>
@@ -3423,7 +3573,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>121</v>
       </c>
@@ -3431,7 +3581,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>130</v>
       </c>
@@ -3439,7 +3589,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>131</v>
       </c>
@@ -3447,7 +3597,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>132</v>
       </c>
@@ -3455,7 +3605,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>133</v>
       </c>
@@ -3463,7 +3613,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>134</v>
       </c>
@@ -3471,7 +3621,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>135</v>
       </c>
@@ -3479,7 +3629,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>136</v>
       </c>
@@ -3487,7 +3637,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>137</v>
       </c>
@@ -3495,7 +3645,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>138</v>
       </c>
@@ -3503,7 +3653,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>139</v>
       </c>
@@ -3511,7 +3661,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>140</v>
       </c>
@@ -3519,7 +3669,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>141</v>
       </c>
@@ -3527,7 +3677,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>144</v>
       </c>
@@ -3535,7 +3685,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>145</v>
       </c>
@@ -3543,7 +3693,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>150</v>
       </c>
@@ -3551,7 +3701,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>153</v>
       </c>
@@ -3559,7 +3709,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>154</v>
       </c>
@@ -3567,7 +3717,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>155</v>
       </c>
@@ -3575,7 +3725,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>156</v>
       </c>
@@ -3583,7 +3733,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>157</v>
       </c>
@@ -3591,7 +3741,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>158</v>
       </c>
@@ -3599,7 +3749,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>159</v>
       </c>
@@ -3607,7 +3757,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
         <v>160</v>
       </c>
@@ -3615,7 +3765,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>161</v>
       </c>
@@ -3623,7 +3773,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
         <v>162</v>
       </c>
@@ -3631,7 +3781,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>163</v>
       </c>
@@ -3639,7 +3789,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>164</v>
       </c>
@@ -3647,7 +3797,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
         <v>165</v>
       </c>
@@ -3655,7 +3805,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>166</v>
       </c>
@@ -3663,7 +3813,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
         <v>167</v>
       </c>
@@ -3671,7 +3821,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" s="4" t="s">
         <v>168</v>
       </c>
@@ -3679,7 +3829,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>169</v>
       </c>
@@ -3687,7 +3837,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
         <v>170</v>
       </c>
@@ -3695,7 +3845,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
         <v>171</v>
       </c>
@@ -3703,7 +3853,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
         <v>172</v>
       </c>
@@ -3711,7 +3861,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
         <v>173</v>
       </c>
@@ -3719,7 +3869,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>174</v>
       </c>
@@ -3727,7 +3877,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
         <v>175</v>
       </c>
@@ -3735,7 +3885,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
         <v>176</v>
       </c>
@@ -3743,7 +3893,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
         <v>11</v>
       </c>
@@ -3751,7 +3901,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
         <v>177</v>
       </c>
@@ -3759,7 +3909,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>178</v>
       </c>
@@ -3767,7 +3917,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>179</v>
       </c>
@@ -3775,7 +3925,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
         <v>180</v>
       </c>
@@ -3783,7 +3933,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" s="4" t="s">
         <v>181</v>
       </c>
@@ -3791,7 +3941,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" s="6" t="s">
         <v>182</v>
       </c>
@@ -3799,7 +3949,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" s="6" t="s">
         <v>183</v>
       </c>
@@ -3807,7 +3957,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
         <v>184</v>
       </c>
@@ -3815,7 +3965,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
         <v>185</v>
       </c>
@@ -3823,7 +3973,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" s="6" t="s">
         <v>186</v>
       </c>
@@ -3831,7 +3981,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
         <v>318</v>
       </c>
@@ -3839,7 +3989,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" s="6" t="s">
         <v>319</v>
       </c>
@@ -3847,7 +3997,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>320</v>
       </c>
@@ -3855,7 +4005,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
         <v>321</v>
       </c>
@@ -3863,7 +4013,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
         <v>38</v>
       </c>
@@ -3871,7 +4021,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" s="4" t="s">
         <v>322</v>
       </c>
@@ -3879,7 +4029,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" s="4" t="s">
         <v>323</v>
       </c>
@@ -3887,7 +4037,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" s="4" t="s">
         <v>324</v>
       </c>
@@ -3895,7 +4045,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A135" s="4" t="s">
         <v>325</v>
       </c>
@@ -3903,7 +4053,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A136" s="4" t="s">
         <v>326</v>
       </c>
@@ -3911,7 +4061,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
         <v>327</v>
       </c>
@@ -3919,7 +4069,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
         <v>328</v>
       </c>
@@ -3927,7 +4077,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" s="4" t="s">
         <v>329</v>
       </c>
@@ -3935,7 +4085,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" s="4" t="s">
         <v>339</v>
       </c>
@@ -3943,7 +4093,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" s="4" t="s">
         <v>340</v>
       </c>
@@ -3951,7 +4101,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" s="4" t="s">
         <v>341</v>
       </c>
@@ -3959,7 +4109,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" s="4" t="s">
         <v>342</v>
       </c>
@@ -3967,7 +4117,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" s="4" t="s">
         <v>343</v>
       </c>
@@ -3975,7 +4125,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A145" s="4" t="s">
         <v>344</v>
       </c>
@@ -3983,7 +4133,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" s="4" t="s">
         <v>345</v>
       </c>
@@ -3991,7 +4141,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A147" s="4" t="s">
         <v>346</v>
       </c>
@@ -3999,7 +4149,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A148" s="4" t="s">
         <v>347</v>
       </c>
@@ -4007,7 +4157,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A149" s="4" t="s">
         <v>348</v>
       </c>
@@ -4015,7 +4165,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A150" s="4" t="s">
         <v>349</v>
       </c>
@@ -4023,7 +4173,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A151" s="4" t="s">
         <v>88</v>
       </c>
@@ -4031,7 +4181,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
         <v>350</v>
       </c>
@@ -4039,7 +4189,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
         <v>351</v>
       </c>
@@ -4047,7 +4197,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
         <v>352</v>
       </c>
@@ -4055,7 +4205,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
         <v>353</v>
       </c>
@@ -4063,7 +4213,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
         <v>354</v>
       </c>
@@ -4071,7 +4221,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A157" s="4" t="s">
         <v>355</v>
       </c>
@@ -4079,7 +4229,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
         <v>376</v>
       </c>
@@ -4087,7 +4237,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A159" s="4" t="s">
         <v>377</v>
       </c>
@@ -4095,7 +4245,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A160" s="4" t="s">
         <v>378</v>
       </c>
@@ -4103,7 +4253,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
         <v>380</v>
       </c>
@@ -4111,7 +4261,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
         <v>382</v>
       </c>
@@ -4119,7 +4269,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
         <v>384</v>
       </c>
@@ -4127,7 +4277,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
         <v>386</v>
       </c>
@@ -4135,7 +4285,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A165" s="4" t="s">
         <v>388</v>
       </c>
@@ -4143,7 +4293,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A166" s="4" t="s">
         <v>390</v>
       </c>
@@ -4151,7 +4301,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A167" s="4" t="s">
         <v>392</v>
       </c>
@@ -4159,7 +4309,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A168" s="4" t="s">
         <v>394</v>
       </c>
@@ -4167,7 +4317,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A169" s="4" t="s">
         <v>396</v>
       </c>
@@ -4175,7 +4325,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A170" s="4" t="s">
         <v>398</v>
       </c>
@@ -4183,7 +4333,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A171" s="4" t="s">
         <v>400</v>
       </c>
@@ -4191,7 +4341,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A172" s="4" t="s">
         <v>402</v>
       </c>
@@ -4199,7 +4349,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A173" s="4" t="s">
         <v>404</v>
       </c>
@@ -4207,7 +4357,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A174" s="4" t="s">
         <v>406</v>
       </c>
@@ -4215,7 +4365,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A175" s="4" t="s">
         <v>408</v>
       </c>
@@ -4223,7 +4373,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A176" s="4" t="s">
         <v>410</v>
       </c>
@@ -4231,7 +4381,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A177" s="4" t="s">
         <v>412</v>
       </c>
@@ -4239,7 +4389,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A178" s="4" t="s">
         <v>414</v>
       </c>
@@ -4247,7 +4397,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A179" s="4" t="s">
         <v>416</v>
       </c>
@@ -4255,7 +4405,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A180" s="4" t="s">
         <v>418</v>
       </c>
@@ -4263,7 +4413,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A181" s="4" t="s">
         <v>420</v>
       </c>
@@ -4271,7 +4421,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A182" s="4" t="s">
         <v>422</v>
       </c>
@@ -4279,7 +4429,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A183" s="4" t="s">
         <v>424</v>
       </c>
@@ -4287,7 +4437,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A184" s="4" t="s">
         <v>426</v>
       </c>
@@ -4295,7 +4445,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A185" s="4" t="s">
         <v>428</v>
       </c>
@@ -4303,7 +4453,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A186" s="4" t="s">
         <v>430</v>
       </c>
@@ -4311,7 +4461,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A187" s="4" t="s">
         <v>432</v>
       </c>
@@ -4319,7 +4469,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A188" s="4" t="s">
         <v>434</v>
       </c>
@@ -4327,7 +4477,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A189" s="4" t="s">
         <v>436</v>
       </c>
@@ -4335,7 +4485,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A190" s="4" t="s">
         <v>438</v>
       </c>
@@ -4343,7 +4493,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A191" s="4" t="s">
         <v>440</v>
       </c>
@@ -4351,7 +4501,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A192" s="4" t="s">
         <v>442</v>
       </c>
@@ -4359,7 +4509,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A193" s="4" t="s">
         <v>444</v>
       </c>
@@ -4367,7 +4517,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A194" s="4" t="s">
         <v>446</v>
       </c>
@@ -4375,7 +4525,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A195" s="4" t="s">
         <v>448</v>
       </c>
@@ -4383,7 +4533,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A196" s="4" t="s">
         <v>450</v>
       </c>
@@ -4391,7 +4541,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A197" s="4" t="s">
         <v>452</v>
       </c>
@@ -4399,7 +4549,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A198" s="4" t="s">
         <v>454</v>
       </c>
@@ -4407,7 +4557,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A199" s="4" t="s">
         <v>456</v>
       </c>
@@ -4415,7 +4565,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A200" s="4" t="s">
         <v>458</v>
       </c>
@@ -4423,7 +4573,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A201" s="4" t="s">
         <v>460</v>
       </c>
@@ -4431,7 +4581,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A202" s="4" t="s">
         <v>462</v>
       </c>
@@ -4439,7 +4589,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A203" s="4" t="s">
         <v>464</v>
       </c>
@@ -4447,7 +4597,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A204" s="4" t="s">
         <v>465</v>
       </c>
@@ -4455,7 +4605,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A205" s="4" t="s">
         <v>467</v>
       </c>
@@ -4463,7 +4613,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A206" s="4" t="s">
         <v>469</v>
       </c>
@@ -4471,7 +4621,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A207" s="4" t="s">
         <v>471</v>
       </c>
@@ -4479,7 +4629,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A208" s="4" t="s">
         <v>473</v>
       </c>
@@ -4487,7 +4637,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A209" s="4" t="s">
         <v>475</v>
       </c>
@@ -4495,7 +4645,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A210" s="4" t="s">
         <v>477</v>
       </c>
@@ -4503,7 +4653,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A211" s="4" t="s">
         <v>479</v>
       </c>
@@ -4511,7 +4661,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A212" s="4" t="s">
         <v>481</v>
       </c>
@@ -4519,7 +4669,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A213" s="4" t="s">
         <v>483</v>
       </c>
@@ -4527,7 +4677,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A214" s="4" t="s">
         <v>485</v>
       </c>
@@ -4535,7 +4685,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A215" s="4" t="s">
         <v>487</v>
       </c>
@@ -4543,7 +4693,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A216" s="4" t="s">
         <v>489</v>
       </c>
@@ -4551,7 +4701,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A217" s="4" t="s">
         <v>491</v>
       </c>
@@ -4559,7 +4709,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A218" s="4" t="s">
         <v>493</v>
       </c>
@@ -4567,7 +4717,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A219" s="4" t="s">
         <v>495</v>
       </c>
@@ -4575,7 +4725,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A220" s="4" t="s">
         <v>497</v>
       </c>
@@ -4583,7 +4733,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A221" s="4" t="s">
         <v>499</v>
       </c>
@@ -4591,7 +4741,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A222" s="4" t="s">
         <v>501</v>
       </c>
@@ -4599,7 +4749,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A223" s="4" t="s">
         <v>503</v>
       </c>
@@ -4607,7 +4757,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A224" s="4" t="s">
         <v>505</v>
       </c>
@@ -4615,7 +4765,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A225" s="4" t="s">
         <v>507</v>
       </c>
@@ -4623,7 +4773,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A226" s="4" t="s">
         <v>25</v>
       </c>
@@ -4631,7 +4781,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A227" s="4" t="s">
         <v>58</v>
       </c>
@@ -4639,7 +4789,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A228" s="4" t="s">
         <v>88</v>
       </c>
@@ -4647,7 +4797,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A229" s="4" t="s">
         <v>152</v>
       </c>
@@ -4655,7 +4805,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A230" s="4" t="s">
         <v>512</v>
       </c>
@@ -4663,7 +4813,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A231" s="4" t="s">
         <v>514</v>
       </c>
@@ -4671,7 +4821,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A232" s="4" t="s">
         <v>21</v>
       </c>
@@ -4679,7 +4829,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A233" s="4" t="s">
         <v>30</v>
       </c>
@@ -4687,7 +4837,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A234" s="4" t="s">
         <v>518</v>
       </c>
@@ -4695,7 +4845,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A235" s="4" t="s">
         <v>54</v>
       </c>
@@ -4703,7 +4853,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A236" s="4" t="s">
         <v>65</v>
       </c>
@@ -4711,7 +4861,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A237" s="4" t="s">
         <v>67</v>
       </c>
@@ -4719,7 +4869,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A238" s="4" t="s">
         <v>80</v>
       </c>
@@ -4727,7 +4877,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A239" s="4" t="s">
         <v>82</v>
       </c>
@@ -4735,7 +4885,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A240" s="4" t="s">
         <v>88</v>
       </c>
@@ -4743,7 +4893,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A241" s="4" t="s">
         <v>96</v>
       </c>
@@ -4751,7 +4901,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A242" s="4" t="s">
         <v>100</v>
       </c>
@@ -4759,7 +4909,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A243" s="4" t="s">
         <v>111</v>
       </c>
@@ -4767,7 +4917,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A244" s="4" t="s">
         <v>129</v>
       </c>
@@ -4775,7 +4925,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A245" s="4" t="s">
         <v>143</v>
       </c>
@@ -4783,7 +4933,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A246" s="4" t="s">
         <v>147</v>
       </c>
@@ -4791,7 +4941,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A247" s="4" t="s">
         <v>149</v>
       </c>
@@ -4799,7 +4949,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A248" s="4" t="s">
         <v>152</v>
       </c>
@@ -4807,7 +4957,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A249" s="4" t="s">
         <v>188</v>
       </c>
@@ -4815,7 +4965,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A250" s="4" t="s">
         <v>533</v>
       </c>
@@ -4823,7 +4973,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A251" s="4" t="s">
         <v>535</v>
       </c>
@@ -4831,7 +4981,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A252" s="4" t="s">
         <v>537</v>
       </c>
@@ -4839,7 +4989,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A253" s="4" t="s">
         <v>539</v>
       </c>
@@ -4847,7 +4997,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A254" s="4" t="s">
         <v>541</v>
       </c>
@@ -4855,7 +5005,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A255" s="4" t="s">
         <v>543</v>
       </c>
@@ -4863,7 +5013,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A256" s="4" t="s">
         <v>545</v>
       </c>
@@ -4871,7 +5021,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A257" s="4" t="s">
         <v>547</v>
       </c>
@@ -4879,7 +5029,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A258" s="4" t="s">
         <v>549</v>
       </c>
@@ -4887,7 +5037,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A259" s="4" t="s">
         <v>551</v>
       </c>
@@ -4895,7 +5045,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A260" s="4" t="s">
         <v>553</v>
       </c>
@@ -4903,7 +5053,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A261" s="4" t="s">
         <v>555</v>
       </c>
@@ -4911,7 +5061,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A262" s="4" t="s">
         <v>507</v>
       </c>
@@ -4919,7 +5069,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A263" s="4" t="s">
         <v>558</v>
       </c>
@@ -4927,7 +5077,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A264" s="4" t="s">
         <v>560</v>
       </c>
@@ -4935,7 +5085,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A265" s="4" t="s">
         <v>562</v>
       </c>
@@ -4943,7 +5093,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A266" s="4" t="s">
         <v>564</v>
       </c>
@@ -4951,7 +5101,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A267" s="4" t="s">
         <v>566</v>
       </c>
@@ -4959,7 +5109,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A268" s="4" t="s">
         <v>568</v>
       </c>
@@ -4967,7 +5117,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A269" s="4" t="s">
         <v>570</v>
       </c>
@@ -4975,7 +5125,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A270" s="4" t="s">
         <v>572</v>
       </c>
@@ -4983,7 +5133,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A271" s="4" t="s">
         <v>574</v>
       </c>
@@ -4991,7 +5141,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A272" s="4" t="s">
         <v>576</v>
       </c>
@@ -4999,7 +5149,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A273" s="4" t="s">
         <v>533</v>
       </c>
@@ -5007,7 +5157,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A274" s="4" t="s">
         <v>577</v>
       </c>
@@ -5015,7 +5165,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A275" s="4" t="s">
         <v>579</v>
       </c>
@@ -5023,7 +5173,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A276" s="4" t="s">
         <v>581</v>
       </c>
@@ -5031,7 +5181,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A277" s="4" t="s">
         <v>583</v>
       </c>
@@ -5039,7 +5189,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A278" s="4" t="s">
         <v>585</v>
       </c>
@@ -5047,7 +5197,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A279" s="4" t="s">
         <v>587</v>
       </c>
@@ -5055,7 +5205,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A280" s="4" t="s">
         <v>589</v>
       </c>
@@ -5063,7 +5213,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A281" s="4" t="s">
         <v>591</v>
       </c>
@@ -5071,7 +5221,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A282" s="4" t="s">
         <v>593</v>
       </c>
@@ -5079,7 +5229,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A283" s="4" t="s">
         <v>595</v>
       </c>
@@ -5087,7 +5237,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A284" s="4" t="s">
         <v>597</v>
       </c>
@@ -5095,7 +5245,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A285" s="4" t="s">
         <v>599</v>
       </c>
@@ -5103,7 +5253,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A286" s="4" t="s">
         <v>601</v>
       </c>
@@ -5111,7 +5261,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A287" s="4" t="s">
         <v>603</v>
       </c>
@@ -5119,7 +5269,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A288" s="4" t="s">
         <v>605</v>
       </c>
@@ -5127,7 +5277,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A289" s="4" t="s">
         <v>607</v>
       </c>
@@ -5135,7 +5285,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A290" s="4" t="s">
         <v>609</v>
       </c>
@@ -5143,7 +5293,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A291" s="4" t="s">
         <v>611</v>
       </c>
@@ -5151,7 +5301,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A292" s="4" t="s">
         <v>562</v>
       </c>
@@ -5159,7 +5309,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A293" s="4" t="s">
         <v>613</v>
       </c>
@@ -5167,7 +5317,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A294" s="4" t="s">
         <v>615</v>
       </c>
@@ -5175,7 +5325,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A295" s="4" t="s">
         <v>599</v>
       </c>
@@ -5183,7 +5333,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A296" s="4" t="s">
         <v>617</v>
       </c>
@@ -5191,7 +5341,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A297" s="4" t="s">
         <v>619</v>
       </c>
@@ -5199,7 +5349,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A298" s="4" t="s">
         <v>621</v>
       </c>
@@ -5207,7 +5357,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A299" s="4" t="s">
         <v>623</v>
       </c>
@@ -5215,7 +5365,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A300" s="4" t="s">
         <v>625</v>
       </c>
@@ -5223,7 +5373,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A301" s="4" t="s">
         <v>627</v>
       </c>
@@ -5231,7 +5381,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A302" s="4" t="s">
         <v>629</v>
       </c>
@@ -5239,7 +5389,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A303" s="4" t="s">
         <v>631</v>
       </c>
@@ -5247,7 +5397,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A304" s="4" t="s">
         <v>633</v>
       </c>
@@ -5255,7 +5405,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A305" s="4" t="s">
         <v>635</v>
       </c>
@@ -5263,7 +5413,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A306" s="4" t="s">
         <v>637</v>
       </c>
@@ -5271,7 +5421,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A307" s="4" t="s">
         <v>639</v>
       </c>
@@ -5279,7 +5429,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A308" s="4" t="s">
         <v>641</v>
       </c>
@@ -5287,7 +5437,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A309" s="4" t="s">
         <v>643</v>
       </c>
@@ -5295,7 +5445,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A310" s="4" t="s">
         <v>645</v>
       </c>
@@ -5303,7 +5453,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A311" s="4" t="s">
         <v>589</v>
       </c>
@@ -5311,7 +5461,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A312" s="4" t="s">
         <v>647</v>
       </c>
@@ -5319,7 +5469,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A313" s="4" t="s">
         <v>67</v>
       </c>
@@ -5327,7 +5477,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A314" s="4" t="s">
         <v>649</v>
       </c>
@@ -5335,7 +5485,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A315" s="4" t="s">
         <v>651</v>
       </c>
@@ -5343,7 +5493,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A316" s="4" t="s">
         <v>653</v>
       </c>
@@ -5351,7 +5501,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A317" s="4" t="s">
         <v>655</v>
       </c>
@@ -5359,7 +5509,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A318" s="4" t="s">
         <v>657</v>
       </c>
@@ -5367,7 +5517,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A319" s="4" t="s">
         <v>659</v>
       </c>
@@ -5375,7 +5525,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A320" s="4" t="s">
         <v>661</v>
       </c>
@@ -5383,7 +5533,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A321" s="4" t="s">
         <v>663</v>
       </c>
@@ -5391,7 +5541,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A322" s="4" t="s">
         <v>665</v>
       </c>
@@ -5399,7 +5549,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A323" s="4" t="s">
         <v>666</v>
       </c>
@@ -5407,7 +5557,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A324" s="4" t="s">
         <v>668</v>
       </c>
@@ -5415,7 +5565,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A325" s="4" t="s">
         <v>670</v>
       </c>
@@ -5423,7 +5573,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A326" s="4" t="s">
         <v>672</v>
       </c>
@@ -5431,7 +5581,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A327" s="4" t="s">
         <v>674</v>
       </c>
@@ -5439,7 +5589,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A328" s="4" t="s">
         <v>676</v>
       </c>
@@ -5447,7 +5597,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A329" s="4" t="s">
         <v>678</v>
       </c>
@@ -5455,7 +5605,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A330" s="4" t="s">
         <v>680</v>
       </c>
@@ -5463,7 +5613,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A331" s="4" t="s">
         <v>682</v>
       </c>
@@ -5471,7 +5621,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A332" s="4" t="s">
         <v>684</v>
       </c>
@@ -5479,7 +5629,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A333" s="4" t="s">
         <v>686</v>
       </c>
@@ -5487,7 +5637,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A334" s="4" t="s">
         <v>688</v>
       </c>
@@ -5495,7 +5645,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A335" s="4" t="s">
         <v>619</v>
       </c>
@@ -5503,7 +5653,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="336" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A336" s="4" t="s">
         <v>690</v>
       </c>
@@ -5511,7 +5661,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="337" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A337" s="4" t="s">
         <v>692</v>
       </c>
@@ -5519,7 +5669,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="338" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A338" s="4" t="s">
         <v>621</v>
       </c>
@@ -5527,7 +5677,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="339" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A339" s="4" t="s">
         <v>694</v>
       </c>
@@ -5535,7 +5685,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="340" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A340" s="4" t="s">
         <v>696</v>
       </c>
@@ -5543,7 +5693,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="341" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A341" s="4" t="s">
         <v>698</v>
       </c>
@@ -5551,7 +5701,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="342" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A342" s="4" t="s">
         <v>700</v>
       </c>
@@ -5559,7 +5709,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="343" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A343" s="4" t="s">
         <v>702</v>
       </c>
@@ -5567,7 +5717,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="344" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A344" s="4" t="s">
         <v>704</v>
       </c>
@@ -5575,7 +5725,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="345" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A345" s="4" t="s">
         <v>706</v>
       </c>
@@ -5583,7 +5733,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="346" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A346" s="4" t="s">
         <v>708</v>
       </c>
@@ -5591,7 +5741,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="347" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A347" s="4" t="s">
         <v>710</v>
       </c>
@@ -5599,7 +5749,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="348" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A348" s="4" t="s">
         <v>712</v>
       </c>
@@ -5607,7 +5757,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="349" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A349" s="4" t="s">
         <v>714</v>
       </c>
@@ -5615,7 +5765,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="350" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A350" s="4" t="s">
         <v>716</v>
       </c>
@@ -5623,7 +5773,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="351" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A351" s="4" t="s">
         <v>718</v>
       </c>
@@ -5631,7 +5781,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="352" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A352" s="4" t="s">
         <v>720</v>
       </c>
@@ -5639,7 +5789,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="353" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A353" s="4" t="s">
         <v>603</v>
       </c>
@@ -5647,7 +5797,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="354" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A354" s="4" t="s">
         <v>577</v>
       </c>
@@ -5655,7 +5805,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="355" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A355" s="4" t="s">
         <v>722</v>
       </c>
@@ -5663,7 +5813,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="356" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A356" s="4" t="s">
         <v>724</v>
       </c>
@@ -5671,7 +5821,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="357" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A357" s="4" t="s">
         <v>726</v>
       </c>
@@ -5679,7 +5829,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="358" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A358" s="4" t="s">
         <v>728</v>
       </c>
@@ -5687,7 +5837,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="359" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A359" s="4" t="s">
         <v>730</v>
       </c>
@@ -5695,7 +5845,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="360" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A360" s="4" t="s">
         <v>627</v>
       </c>
@@ -5703,7 +5853,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="361" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A361" s="4" t="s">
         <v>733</v>
       </c>
@@ -5711,7 +5861,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="362" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A362" s="4" t="s">
         <v>633</v>
       </c>
@@ -5719,7 +5869,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="363" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A363" s="4" t="s">
         <v>639</v>
       </c>
@@ -5727,7 +5877,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="364" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A364" s="4" t="s">
         <v>735</v>
       </c>
@@ -5735,7 +5885,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="365" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A365" s="4" t="s">
         <v>737</v>
       </c>
@@ -5743,7 +5893,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="366" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A366" s="4" t="s">
         <v>738</v>
       </c>
@@ -5751,7 +5901,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="367" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A367" s="4" t="s">
         <v>740</v>
       </c>
@@ -5759,7 +5909,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="368" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A368" s="4" t="s">
         <v>742</v>
       </c>
@@ -5767,7 +5917,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="369" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A369" s="4" t="s">
         <v>744</v>
       </c>
@@ -5775,7 +5925,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="370" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A370" s="4" t="s">
         <v>746</v>
       </c>
@@ -5783,7 +5933,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="371" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A371" s="4" t="s">
         <v>748</v>
       </c>
@@ -5791,7 +5941,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="372" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A372" s="4" t="s">
         <v>750</v>
       </c>
@@ -5799,7 +5949,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="373" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A373" s="4" t="s">
         <v>752</v>
       </c>
@@ -5807,7 +5957,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="374" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A374" s="4" t="s">
         <v>572</v>
       </c>
@@ -5815,7 +5965,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="375" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A375" s="4" t="s">
         <v>754</v>
       </c>
@@ -5823,7 +5973,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="376" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A376" s="4" t="s">
         <v>67</v>
       </c>
@@ -5831,7 +5981,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="377" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A377" s="4" t="s">
         <v>653</v>
       </c>
@@ -5839,7 +5989,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="378" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A378" s="4" t="s">
         <v>756</v>
       </c>
@@ -5847,7 +5997,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="379" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A379" s="4" t="s">
         <v>758</v>
       </c>
@@ -5855,7 +6005,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="380" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A380" s="4" t="s">
         <v>760</v>
       </c>
@@ -5863,12 +6013,212 @@
         <v>761</v>
       </c>
     </row>
-    <row r="381" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A381" s="4" t="s">
         <v>762</v>
       </c>
       <c r="B381" s="8" t="s">
         <v>763</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A382" t="s">
+        <v>764</v>
+      </c>
+      <c r="B382" s="8" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A383" t="s">
+        <v>766</v>
+      </c>
+      <c r="B383" s="8" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A384" t="s">
+        <v>768</v>
+      </c>
+      <c r="B384" s="8" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A385" t="s">
+        <v>770</v>
+      </c>
+      <c r="B385" s="8" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A386" t="s">
+        <v>772</v>
+      </c>
+      <c r="B386" s="8" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A387" t="s">
+        <v>774</v>
+      </c>
+      <c r="B387" s="8" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A388" t="s">
+        <v>776</v>
+      </c>
+      <c r="B388" s="8" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A389" t="s">
+        <v>778</v>
+      </c>
+      <c r="B389" s="8" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A390" t="s">
+        <v>780</v>
+      </c>
+      <c r="B390" s="8" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A391" t="s">
+        <v>782</v>
+      </c>
+      <c r="B391" s="8" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A392" t="s">
+        <v>784</v>
+      </c>
+      <c r="B392" s="8" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A393" t="s">
+        <v>786</v>
+      </c>
+      <c r="B393" s="8" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A394" t="s">
+        <v>788</v>
+      </c>
+      <c r="B394" s="8" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A395" t="s">
+        <v>790</v>
+      </c>
+      <c r="B395" s="8" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A396" t="s">
+        <v>792</v>
+      </c>
+      <c r="B396" s="8" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A397" t="s">
+        <v>794</v>
+      </c>
+      <c r="B397" s="8" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A398" t="s">
+        <v>796</v>
+      </c>
+      <c r="B398" s="8" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A399" t="s">
+        <v>798</v>
+      </c>
+      <c r="B399" s="8" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A400" t="s">
+        <v>800</v>
+      </c>
+      <c r="B400" s="8" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A401" t="s">
+        <v>802</v>
+      </c>
+      <c r="B401" s="8" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A402" t="s">
+        <v>804</v>
+      </c>
+      <c r="B402" s="8" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A403" t="s">
+        <v>806</v>
+      </c>
+      <c r="B403" s="8" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A404" t="s">
+        <v>808</v>
+      </c>
+      <c r="B404" s="8" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A405" t="s">
+        <v>810</v>
+      </c>
+      <c r="B405" s="8" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A406" t="s">
+        <v>812</v>
+      </c>
+      <c r="B406" s="8" t="s">
+        <v>813</v>
       </c>
     </row>
   </sheetData>
@@ -6097,21 +6447,22 @@
     <hyperlink ref="B223" r:id="rId222" xr:uid="{18E1B368-34D0-4DAD-9143-1F342221F5FD}"/>
     <hyperlink ref="B224" r:id="rId223" xr:uid="{539E6B87-0B3A-4A6D-BEE7-156C0B6E8621}"/>
     <hyperlink ref="B225" r:id="rId224" xr:uid="{40B35693-E051-4A9A-8155-D184C284834F}"/>
+    <hyperlink ref="A404" r:id="rId225" display="https://thesisrationale.substack.com/" xr:uid="{29A2B7B1-3503-4E6C-88B0-32AE47FB9618}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId225"/>
+  <pageSetup orientation="portrait" r:id="rId226"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C24231E-54D9-429F-828F-B65126FC6988}">
   <dimension ref="B2:L24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="29.90625" customWidth="1"/>
+    <col min="3" max="3" width="29.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>15</v>
       </c>
@@ -6125,7 +6476,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -6142,7 +6493,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>2</v>
       </c>
@@ -6153,7 +6504,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>3</v>
       </c>
@@ -6164,7 +6515,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>4</v>
       </c>
@@ -6175,7 +6526,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>5</v>
       </c>
@@ -6186,7 +6537,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>6</v>
       </c>
@@ -6197,7 +6548,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7</v>
       </c>
@@ -6208,7 +6559,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>8</v>
       </c>
@@ -6219,7 +6570,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>9</v>
       </c>
@@ -6230,7 +6581,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>10</v>
       </c>
@@ -6241,7 +6592,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>11</v>
       </c>
@@ -6252,7 +6603,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>12</v>
       </c>
@@ -6263,7 +6614,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>13</v>
       </c>
@@ -6274,7 +6625,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>14</v>
       </c>
@@ -6285,7 +6636,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>15</v>
       </c>
@@ -6296,7 +6647,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>16</v>
       </c>
@@ -6307,7 +6658,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>17</v>
       </c>
@@ -6318,7 +6669,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>18</v>
       </c>
@@ -6329,7 +6680,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>19</v>
       </c>
@@ -6340,7 +6691,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>20</v>
       </c>
@@ -6351,7 +6702,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>21</v>
       </c>
@@ -6362,7 +6713,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>22</v>
       </c>

</xml_diff>